<commit_message>
Fixed a major agg_metrics_test.rds issue and downstream impacts. - Corrected predict-only folder handling - Repaired corrupted run_predict function in utils.R - Added LoadandPredict.R supporting both Stateful and Stateless execution - New artifacts folder creation for LoadandPredict runs
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>204</v>
+        <v>230</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>173</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>346</v>
+        <v>515</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>27</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.73333333</v>
+        <v>0.99333333</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.54111406</v>
+        <v>0.98290598</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.88311688</v>
+        <v>0.995671</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.67105263</v>
+        <v>0.98924731</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.833333333333333</v>
+        <v>0.998666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.77319587628866</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.649350649350649</v>
+        <v>0.995670995670996</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.705882352941177</v>
+        <v>0.997830802603037</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.79</v>
+        <v>0.51</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.880130787645239</v>
+        <v>0.999908248463162</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
release: 5.6.5 — fresh push for LoadandPredict and cleaned up train_with_l2_regulization
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>230</v>
+        <v>215</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>236</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>515</v>
+        <v>283</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>1</v>
+        <v>16</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.99333333</v>
+        <v>0.664</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.98290598</v>
+        <v>0.4767184</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.995671</v>
+        <v>0.93073593</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.98924731</v>
+        <v>0.63049853</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.998666666666667</v>
+        <v>0.82</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>1</v>
+        <v>0.766666666666667</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.995670995670996</v>
+        <v>0.597402597402597</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.997830802603037</v>
+        <v>0.671532846715329</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.51</v>
+        <v>0.77</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.999908248463162</v>
+        <v>0.875409754022471</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
## SCENARIO B: Single-run, MULTI-MODEL (no ensemble) - do_ensemble <- FALSE - num_networks <- 4L (multi-model single instance) - num_temp_iterations <- 0L - Verified working for SingleRuns in v5.6.7
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>215</v>
+        <v>226</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>236</v>
+        <v>7</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>283</v>
+        <v>512</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>16</v>
+        <v>5</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.664</v>
+        <v>0.984</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.4767184</v>
+        <v>0.96995708</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.93073593</v>
+        <v>0.97835498</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.63049853</v>
+        <v>0.97413793</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.82</v>
+        <v>0.985333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.766666666666667</v>
+        <v>0.966101694915254</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.597402597402597</v>
+        <v>0.987012987012987</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.671532846715329</v>
+        <v>0.97644539614561</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.77</v>
+        <v>0.49</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.875409754022471</v>
+        <v>0.998744672155077</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v5.6.8 — clean ensembles and single runs for num_networks >= 1, and LoadAndPredict now matches test.rds objects. Did not test seeds too much here but they probably work.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>226</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>7</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>512</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.984</v>
+        <v>0.61466667</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.96995708</v>
+        <v>0.44268775</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.97835498</v>
+        <v>0.96969697</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.97413793</v>
+        <v>0.60786974</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.985333333333333</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.966101694915254</v>
+        <v>0.738197424892704</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.987012987012987</v>
+        <v>0.744588744588745</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.97644539614561</v>
+        <v>0.741379310344828</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.49</v>
+        <v>0.76</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.998744672155077</v>
+        <v>0.886428279491863</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v5.6.10 — grouped performance comments, store_metadata signature/call, and temp-train var
- Updated grouped performance section comments for clarity and consistency.
- Revised store_metadata() call and function signature to align (fixed arg mismatches / clarified names).
- Ensured TEMP training path in TestDESONN.R assigns into a clearly named variable: model_results_temp.
- Minor hygiene: kept prior v5.6.9 behavior intact; no breaking changes to public APIs beyond the aligned signature.

Why:
- Improve readability and reduce confusion in grouped performance reporting.
- Prevent runtime signature/call mismatches in metadata storage.
- Make TEMP train/test flow explicit and self-documenting via model_results_temp.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>224</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>237</v>
+        <v>519</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>231</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.61466667</v>
+        <v>0.692</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.44268775</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.96969697</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.60786974</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.84</v>
+        <v>0.705333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.738197424892704</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.744588744588745</v>
+        <v>0.0432900432900433</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.741379310344828</v>
+        <v>0.0829875518672199</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.76</v>
+        <v>0.43</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.886428279491863</v>
+        <v>0.542301629006831</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v5.6.13 — got SL_NN to work by fixing predict call in DDESONN_predict_eval()
- Fixed .safe_run_predict by removing recursive default arg (no more promise error).
- ML_NN flow unchanged. Now picks predictor safely, passes only valid args,
  normalizes outputs to double matrix, and logs dims/stats.
- .run_predict made mode-aware, checks weights/biases, builds model shell,
  calls predict safely, normalizes output, and keeps ML_NN behavior intact.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>5</v>
+        <v>224</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>282</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>515</v>
+        <v>237</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>226</v>
+        <v>7</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.69333333</v>
+        <v>0.61466667</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.55555556</v>
+        <v>0.44268775</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.02164502</v>
+        <v>0.96969697</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.04166667</v>
+        <v>0.60786974</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.728</v>
+        <v>0.84</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.601503759398496</v>
+        <v>0.738197424892704</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.346320346320346</v>
+        <v>0.744588744588745</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.43956043956044</v>
+        <v>0.741379310344828</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.19</v>
+        <v>0.76</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.646439623318236</v>
+        <v>0.886428279491863</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
6.3.2 Checkpoint — believe things are working again after the whitespace error mess. 6.2.4 to 6.3.1 uncertain effect from whitespace edits, but this is latest stable without that implementation.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>224</v>
+        <v>0</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>282</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>237</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>7</v>
+        <v>2</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.61466667</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.44268775</v>
+        <v>0</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0.96969697</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.60786974</v>
+        <v>0</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.84</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.738197424892704</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0.744588744588745</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.741379310344828</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -803,7 +803,7 @@
         <v>11</v>
       </c>
       <c r="B6" t="n">
-        <v>0.76</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.886428279491863</v>
+        <v>0.5</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
v6.4.1 TestDDESONN.R verified + heart_failure_example learns correctly across auto/single/multi architectures
Summary:
- TestDDESONN.R now confirmed functional and included properly in pushes (previously missed).
- ddesonn_heart_failure_example.R fixed learning behavior across single, multi, and auto architectures.
- Activation functions now accepted as list, vector, single string, or function — normalized before learn/predict.
- Works with all CRAN-compatibility updates; no breaking changes.

Result:
Everything from TestDDESONN.R to heart_failure_example now trains correctly with consistent activation normalization and architecture detection.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.666666666666667</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.666666666666667</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0</v>
+        <v>0.333333333333333</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="6">

</xml_diff>

<commit_message>
v6.6.1 checkpoint: working on DDESONN_mtcars_A-D_examples trainmetrics.rds metrics print
• Example mirrors TestDDESONN.R very cleanly.
• Clearly indicates which scenario (A–D) the user/student is running.
• Consistent trainmetrics.rds output with clear metric prints.
</commit_message>
<xml_diff>
--- a/Rdata_predictions.xlsx
+++ b/Rdata_predictions.xlsx
@@ -679,7 +679,7 @@
         <v>2</v>
       </c>
       <c r="B2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -687,7 +687,7 @@
         <v>3</v>
       </c>
       <c r="B3" t="n">
-        <v>4</v>
+        <v>0</v>
       </c>
     </row>
     <row r="4">
@@ -695,7 +695,7 @@
         <v>4</v>
       </c>
       <c r="B4" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
     </row>
     <row r="5">
@@ -703,7 +703,7 @@
         <v>5</v>
       </c>
       <c r="B5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="6">
@@ -711,7 +711,7 @@
         <v>6</v>
       </c>
       <c r="B6" t="n">
-        <v>0.333333333333333</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="7">
@@ -719,7 +719,7 @@
         <v>7</v>
       </c>
       <c r="B7" t="n">
-        <v>0.333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -727,7 +727,7 @@
         <v>8</v>
       </c>
       <c r="B8" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="9">
@@ -735,7 +735,7 @@
         <v>9</v>
       </c>
       <c r="B9" t="n">
-        <v>0.5</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="10">
@@ -771,7 +771,7 @@
         <v>6</v>
       </c>
       <c r="B2" t="n">
-        <v>0.333333333333333</v>
+        <v>0.833333333333333</v>
       </c>
     </row>
     <row r="3">
@@ -779,7 +779,7 @@
         <v>7</v>
       </c>
       <c r="B3" t="n">
-        <v>0.333333333333333</v>
+        <v>1</v>
       </c>
     </row>
     <row r="4">
@@ -787,7 +787,7 @@
         <v>8</v>
       </c>
       <c r="B4" t="n">
-        <v>1</v>
+        <v>0.5</v>
       </c>
     </row>
     <row r="5">
@@ -795,7 +795,7 @@
         <v>9</v>
       </c>
       <c r="B5" t="n">
-        <v>0.5</v>
+        <v>0.666666666666667</v>
       </c>
     </row>
     <row r="6">
@@ -825,7 +825,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>0.5</v>
+        <v>0.875</v>
       </c>
     </row>
   </sheetData>

</xml_diff>